<commit_message>
Adiciona busca em grade para otimizar os hiperparâmetros da regressão logística, testando diferentes valores de C e class_weight. Melhor configuração encontrada: C=0.5 e class_weight='balanced'. Validação cruzada: 46,25%. Treino médio nos folds: 64,21%. Gap treino-validação: 17,96 p.p.
Gera o relatório grid_top10.csv com os hiperparâmetros testados e seus resultados.
</commit_message>
<xml_diff>
--- a/teste_rotulado.xlsx
+++ b/teste_rotulado.xlsx
@@ -520,7 +520,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -1396,7 +1396,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -1876,7 +1876,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -2476,7 +2476,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -2980,7 +2980,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -3172,7 +3172,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -3436,7 +3436,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -3568,7 +3568,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -3916,7 +3916,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -4060,7 +4060,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -4336,7 +4336,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -4420,7 +4420,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -4516,7 +4516,7 @@
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -4624,7 +4624,7 @@
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -4720,7 +4720,7 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -5032,7 +5032,7 @@
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -5200,7 +5200,7 @@
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -5356,7 +5356,7 @@
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -5608,7 +5608,7 @@
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -5740,7 +5740,7 @@
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -5788,7 +5788,7 @@
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -6124,7 +6124,7 @@
       </c>
       <c r="B475" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -6148,7 +6148,7 @@
       </c>
       <c r="B477" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -6904,7 +6904,7 @@
       </c>
       <c r="B540" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -7288,7 +7288,7 @@
       </c>
       <c r="B572" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -7360,7 +7360,7 @@
       </c>
       <c r="B578" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -7504,7 +7504,7 @@
       </c>
       <c r="B590" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -7636,7 +7636,7 @@
       </c>
       <c r="B601" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -7852,7 +7852,7 @@
       </c>
       <c r="B619" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -8032,7 +8032,7 @@
       </c>
       <c r="B634" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -8464,7 +8464,7 @@
       </c>
       <c r="B670" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -8668,7 +8668,7 @@
       </c>
       <c r="B687" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -9148,7 +9148,7 @@
       </c>
       <c r="B727" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -9268,7 +9268,7 @@
       </c>
       <c r="B737" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -9328,7 +9328,7 @@
       </c>
       <c r="B742" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -9400,7 +9400,7 @@
       </c>
       <c r="B748" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -10216,7 +10216,7 @@
       </c>
       <c r="B816" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -10264,7 +10264,7 @@
       </c>
       <c r="B820" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -10420,7 +10420,7 @@
       </c>
       <c r="B833" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -10492,7 +10492,7 @@
       </c>
       <c r="B839" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -10576,7 +10576,7 @@
       </c>
       <c r="B846" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -10756,7 +10756,7 @@
       </c>
       <c r="B861" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -10900,7 +10900,7 @@
       </c>
       <c r="B873" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -11224,7 +11224,7 @@
       </c>
       <c r="B900" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Amplia o grid search para incluir parâmetros do TF-IDF e da regressão logística, testando ngram_range, min_df, C e class_weight.
Melhor configuração: ngram_range=(1,2), min_df=10, C=0.5 e class_weight='balanced'.
Validação cruzada: 46,30%.
Treino médio nos folds: 64,06%.
Treino final: 63,57%.
Gap treino-validação: 17,76 p.p.
</commit_message>
<xml_diff>
--- a/teste_rotulado.xlsx
+++ b/teste_rotulado.xlsx
@@ -472,7 +472,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -532,7 +532,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -736,7 +736,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -928,7 +928,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1264,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -1612,7 +1612,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -1624,7 +1624,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -1708,7 +1708,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -1732,7 +1732,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -1840,7 +1840,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -1864,7 +1864,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -1876,7 +1876,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -2200,7 +2200,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -2284,7 +2284,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -2356,7 +2356,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -2380,7 +2380,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -2608,7 +2608,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -2824,7 +2824,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -2872,7 +2872,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -3076,7 +3076,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -3148,7 +3148,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -3208,7 +3208,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -3220,7 +3220,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -3232,7 +3232,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -3448,7 +3448,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -3460,7 +3460,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -3472,7 +3472,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -3508,7 +3508,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -3592,7 +3592,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -3616,7 +3616,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -3652,7 +3652,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -3712,7 +3712,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -3724,7 +3724,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -3868,7 +3868,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -4024,7 +4024,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -4048,7 +4048,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -4108,7 +4108,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -4132,7 +4132,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -4168,7 +4168,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -4216,7 +4216,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -4324,7 +4324,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -4336,7 +4336,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -4468,7 +4468,7 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -4516,7 +4516,7 @@
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -4756,7 +4756,7 @@
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -4792,7 +4792,7 @@
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -4924,7 +4924,7 @@
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -4972,7 +4972,7 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -5032,7 +5032,7 @@
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -5320,7 +5320,7 @@
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -5356,7 +5356,7 @@
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -5716,7 +5716,7 @@
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -5788,7 +5788,7 @@
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -5896,7 +5896,7 @@
       </c>
       <c r="B456" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -6028,7 +6028,7 @@
       </c>
       <c r="B467" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -6124,7 +6124,7 @@
       </c>
       <c r="B475" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -6256,7 +6256,7 @@
       </c>
       <c r="B486" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -6352,7 +6352,7 @@
       </c>
       <c r="B494" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -6412,7 +6412,7 @@
       </c>
       <c r="B499" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -6424,7 +6424,7 @@
       </c>
       <c r="B500" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -6472,7 +6472,7 @@
       </c>
       <c r="B504" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -6508,7 +6508,7 @@
       </c>
       <c r="B507" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -6688,7 +6688,7 @@
       </c>
       <c r="B522" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -6724,7 +6724,7 @@
       </c>
       <c r="B525" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -6880,7 +6880,7 @@
       </c>
       <c r="B538" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -6904,7 +6904,7 @@
       </c>
       <c r="B540" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -6964,7 +6964,7 @@
       </c>
       <c r="B545" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -7288,7 +7288,7 @@
       </c>
       <c r="B572" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -7408,7 +7408,7 @@
       </c>
       <c r="B582" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -7780,7 +7780,7 @@
       </c>
       <c r="B613" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -7996,7 +7996,7 @@
       </c>
       <c r="B631" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -8044,7 +8044,7 @@
       </c>
       <c r="B635" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -8128,7 +8128,7 @@
       </c>
       <c r="B642" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -8176,7 +8176,7 @@
       </c>
       <c r="B646" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -8236,7 +8236,7 @@
       </c>
       <c r="B651" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -8248,7 +8248,7 @@
       </c>
       <c r="B652" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -8452,7 +8452,7 @@
       </c>
       <c r="B669" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -8464,7 +8464,7 @@
       </c>
       <c r="B670" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -8584,7 +8584,7 @@
       </c>
       <c r="B680" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -8632,7 +8632,7 @@
       </c>
       <c r="B684" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -8668,7 +8668,7 @@
       </c>
       <c r="B687" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -8800,7 +8800,7 @@
       </c>
       <c r="B698" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -8956,7 +8956,7 @@
       </c>
       <c r="B711" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -8968,7 +8968,7 @@
       </c>
       <c r="B712" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -9088,7 +9088,7 @@
       </c>
       <c r="B722" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -9184,7 +9184,7 @@
       </c>
       <c r="B730" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -9244,7 +9244,7 @@
       </c>
       <c r="B735" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -9268,7 +9268,7 @@
       </c>
       <c r="B737" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -9340,7 +9340,7 @@
       </c>
       <c r="B743" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -9376,7 +9376,7 @@
       </c>
       <c r="B746" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -9496,7 +9496,7 @@
       </c>
       <c r="B756" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -9604,7 +9604,7 @@
       </c>
       <c r="B765" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -9700,7 +9700,7 @@
       </c>
       <c r="B773" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -9712,7 +9712,7 @@
       </c>
       <c r="B774" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -9796,7 +9796,7 @@
       </c>
       <c r="B781" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -9940,7 +9940,7 @@
       </c>
       <c r="B793" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -9964,7 +9964,7 @@
       </c>
       <c r="B795" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -10060,7 +10060,7 @@
       </c>
       <c r="B803" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -10132,7 +10132,7 @@
       </c>
       <c r="B809" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -10156,7 +10156,7 @@
       </c>
       <c r="B811" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -10240,7 +10240,7 @@
       </c>
       <c r="B818" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -10288,7 +10288,7 @@
       </c>
       <c r="B822" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -10300,7 +10300,7 @@
       </c>
       <c r="B823" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -10420,7 +10420,7 @@
       </c>
       <c r="B833" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -10492,7 +10492,7 @@
       </c>
       <c r="B839" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -10552,7 +10552,7 @@
       </c>
       <c r="B844" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -10576,7 +10576,7 @@
       </c>
       <c r="B846" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -10636,7 +10636,7 @@
       </c>
       <c r="B851" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -10684,7 +10684,7 @@
       </c>
       <c r="B855" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -10756,7 +10756,7 @@
       </c>
       <c r="B861" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -10792,7 +10792,7 @@
       </c>
       <c r="B864" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -10864,7 +10864,7 @@
       </c>
       <c r="B870" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -10948,7 +10948,7 @@
       </c>
       <c r="B877" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -10996,7 +10996,7 @@
       </c>
       <c r="B881" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -11008,7 +11008,7 @@
       </c>
       <c r="B882" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -11032,7 +11032,7 @@
       </c>
       <c r="B884" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -11104,7 +11104,7 @@
       </c>
       <c r="B890" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -11224,7 +11224,7 @@
       </c>
       <c r="B900" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adiciona combinação de TF-IDF de palavras e caracteres com regressão logística para avaliar ganho de representação.
Validação cruzada: 46,22%.
Treino médio nos folds: 67,16%.
Treino final: 66,65%.
Gap treino-validação: 20,94 p.p.
</commit_message>
<xml_diff>
--- a/teste_rotulado.xlsx
+++ b/teste_rotulado.xlsx
@@ -472,7 +472,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -520,7 +520,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -532,7 +532,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -724,7 +724,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -844,7 +844,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -928,7 +928,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -1156,7 +1156,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -1324,7 +1324,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -1396,7 +1396,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -1408,7 +1408,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -1636,7 +1636,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -1828,7 +1828,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -1852,7 +1852,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -1876,7 +1876,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -1900,7 +1900,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -1960,7 +1960,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -2284,7 +2284,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -2320,7 +2320,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -2344,7 +2344,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -2356,7 +2356,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -2608,7 +2608,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -2824,7 +2824,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -2944,7 +2944,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -3040,7 +3040,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -3088,7 +3088,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -3124,7 +3124,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -3172,7 +3172,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -3220,7 +3220,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -3232,7 +3232,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -3448,7 +3448,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -3460,7 +3460,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -3472,7 +3472,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -3508,7 +3508,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -3532,7 +3532,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -3568,7 +3568,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -3712,7 +3712,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -3868,7 +3868,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -3904,7 +3904,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -4024,7 +4024,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -4132,7 +4132,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -4216,7 +4216,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -4264,7 +4264,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -4276,7 +4276,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -4480,7 +4480,7 @@
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -4540,7 +4540,7 @@
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -4624,7 +4624,7 @@
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -4756,7 +4756,7 @@
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -4768,7 +4768,7 @@
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -4972,7 +4972,7 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -5032,7 +5032,7 @@
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -5080,7 +5080,7 @@
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -5236,7 +5236,7 @@
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -5248,7 +5248,7 @@
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -5608,7 +5608,7 @@
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -5620,7 +5620,7 @@
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -5716,7 +5716,7 @@
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -5788,7 +5788,7 @@
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -5908,7 +5908,7 @@
       </c>
       <c r="B457" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -5944,7 +5944,7 @@
       </c>
       <c r="B460" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -5980,7 +5980,7 @@
       </c>
       <c r="B463" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -6028,7 +6028,7 @@
       </c>
       <c r="B467" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -6064,7 +6064,7 @@
       </c>
       <c r="B470" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -6160,7 +6160,7 @@
       </c>
       <c r="B478" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -6244,7 +6244,7 @@
       </c>
       <c r="B485" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -6256,7 +6256,7 @@
       </c>
       <c r="B486" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -6268,7 +6268,7 @@
       </c>
       <c r="B487" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -6400,7 +6400,7 @@
       </c>
       <c r="B498" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -6424,7 +6424,7 @@
       </c>
       <c r="B500" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -6688,7 +6688,7 @@
       </c>
       <c r="B522" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -6724,7 +6724,7 @@
       </c>
       <c r="B525" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -6772,7 +6772,7 @@
       </c>
       <c r="B529" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -6784,7 +6784,7 @@
       </c>
       <c r="B530" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -6808,7 +6808,7 @@
       </c>
       <c r="B532" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -6904,7 +6904,7 @@
       </c>
       <c r="B540" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -6976,7 +6976,7 @@
       </c>
       <c r="B546" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -7348,7 +7348,7 @@
       </c>
       <c r="B577" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -7408,7 +7408,7 @@
       </c>
       <c r="B582" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -7636,7 +7636,7 @@
       </c>
       <c r="B601" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -8128,7 +8128,7 @@
       </c>
       <c r="B642" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -8464,7 +8464,7 @@
       </c>
       <c r="B670" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -8488,7 +8488,7 @@
       </c>
       <c r="B672" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -8500,7 +8500,7 @@
       </c>
       <c r="B673" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -8584,7 +8584,7 @@
       </c>
       <c r="B680" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -8668,7 +8668,7 @@
       </c>
       <c r="B687" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -8728,7 +8728,7 @@
       </c>
       <c r="B692" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -8788,7 +8788,7 @@
       </c>
       <c r="B697" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -8800,7 +8800,7 @@
       </c>
       <c r="B698" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -8848,7 +8848,7 @@
       </c>
       <c r="B702" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -8860,7 +8860,7 @@
       </c>
       <c r="B703" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -8968,7 +8968,7 @@
       </c>
       <c r="B712" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -9136,7 +9136,7 @@
       </c>
       <c r="B726" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -9208,7 +9208,7 @@
       </c>
       <c r="B732" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -9376,7 +9376,7 @@
       </c>
       <c r="B746" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -9472,7 +9472,7 @@
       </c>
       <c r="B754" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -9520,7 +9520,7 @@
       </c>
       <c r="B758" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -9652,7 +9652,7 @@
       </c>
       <c r="B769" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -9832,7 +9832,7 @@
       </c>
       <c r="B784" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -9940,7 +9940,7 @@
       </c>
       <c r="B793" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -10072,7 +10072,7 @@
       </c>
       <c r="B804" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -10120,7 +10120,7 @@
       </c>
       <c r="B808" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -10144,7 +10144,7 @@
       </c>
       <c r="B810" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -10216,7 +10216,7 @@
       </c>
       <c r="B816" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -10252,7 +10252,7 @@
       </c>
       <c r="B819" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -10300,7 +10300,7 @@
       </c>
       <c r="B823" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -10420,7 +10420,7 @@
       </c>
       <c r="B833" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -10492,7 +10492,7 @@
       </c>
       <c r="B839" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -10504,7 +10504,7 @@
       </c>
       <c r="B840" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -10552,7 +10552,7 @@
       </c>
       <c r="B844" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -10900,7 +10900,7 @@
       </c>
       <c r="B873" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -10948,7 +10948,7 @@
       </c>
       <c r="B877" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -11032,7 +11032,7 @@
       </c>
       <c r="B884" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -11224,7 +11224,7 @@
       </c>
       <c r="B900" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Removido TF-IDF de caracteres para o aumento da acurácia
</commit_message>
<xml_diff>
--- a/teste_rotulado.xlsx
+++ b/teste_rotulado.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,12 +417,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>resp_text</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>clarity</t>
         </is>
@@ -472,7 +460,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -520,7 +508,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -532,7 +520,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -724,7 +712,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -844,7 +832,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -928,7 +916,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -1132,7 +1120,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -1156,7 +1144,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1204,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -1228,7 +1216,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -1324,7 +1312,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -1396,7 +1384,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -1408,7 +1396,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -1636,7 +1624,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -1828,7 +1816,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -1852,7 +1840,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -1900,7 +1888,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -1912,7 +1900,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -1960,7 +1948,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2128,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -2284,7 +2272,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -2320,7 +2308,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -2344,7 +2332,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -2356,7 +2344,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -2824,7 +2812,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -2944,7 +2932,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -3040,7 +3028,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -3124,7 +3112,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3184,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -3220,7 +3208,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -3232,7 +3220,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -3460,7 +3448,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -3472,7 +3460,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -3508,7 +3496,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -3532,7 +3520,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -3712,7 +3700,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -3904,7 +3892,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -4024,7 +4012,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -4132,7 +4120,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -4216,7 +4204,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -4264,7 +4252,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -4276,7 +4264,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -4540,7 +4528,7 @@
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -4624,7 +4612,7 @@
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -4744,7 +4732,7 @@
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -4756,7 +4744,7 @@
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -4768,7 +4756,7 @@
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -4780,7 +4768,7 @@
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -4972,7 +4960,7 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -5032,7 +5020,7 @@
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -5236,7 +5224,7 @@
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -5248,7 +5236,7 @@
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -5608,7 +5596,7 @@
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -5620,7 +5608,7 @@
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -5716,7 +5704,7 @@
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -5788,7 +5776,7 @@
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -5908,7 +5896,7 @@
       </c>
       <c r="B457" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -5944,7 +5932,7 @@
       </c>
       <c r="B460" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -5980,7 +5968,7 @@
       </c>
       <c r="B463" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -6028,7 +6016,7 @@
       </c>
       <c r="B467" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -6064,7 +6052,7 @@
       </c>
       <c r="B470" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -6160,7 +6148,7 @@
       </c>
       <c r="B478" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -6220,7 +6208,7 @@
       </c>
       <c r="B483" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -6244,7 +6232,7 @@
       </c>
       <c r="B485" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -6256,7 +6244,7 @@
       </c>
       <c r="B486" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -6268,7 +6256,7 @@
       </c>
       <c r="B487" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -6400,7 +6388,7 @@
       </c>
       <c r="B498" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -6424,7 +6412,7 @@
       </c>
       <c r="B500" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -6688,7 +6676,7 @@
       </c>
       <c r="B522" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -6772,7 +6760,7 @@
       </c>
       <c r="B529" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -6784,7 +6772,7 @@
       </c>
       <c r="B530" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -6808,7 +6796,7 @@
       </c>
       <c r="B532" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -6904,7 +6892,7 @@
       </c>
       <c r="B540" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -6976,7 +6964,7 @@
       </c>
       <c r="B546" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -7408,7 +7396,7 @@
       </c>
       <c r="B582" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -7636,7 +7624,7 @@
       </c>
       <c r="B601" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -7864,7 +7852,7 @@
       </c>
       <c r="B620" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -8464,7 +8452,7 @@
       </c>
       <c r="B670" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -8488,7 +8476,7 @@
       </c>
       <c r="B672" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -8500,7 +8488,7 @@
       </c>
       <c r="B673" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -8584,7 +8572,7 @@
       </c>
       <c r="B680" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -8668,7 +8656,7 @@
       </c>
       <c r="B687" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -8728,7 +8716,7 @@
       </c>
       <c r="B692" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -8788,7 +8776,7 @@
       </c>
       <c r="B697" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -8848,7 +8836,7 @@
       </c>
       <c r="B702" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -8860,7 +8848,7 @@
       </c>
       <c r="B703" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -8968,7 +8956,7 @@
       </c>
       <c r="B712" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -9136,7 +9124,7 @@
       </c>
       <c r="B726" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -9208,7 +9196,7 @@
       </c>
       <c r="B732" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -9376,7 +9364,7 @@
       </c>
       <c r="B746" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -9448,7 +9436,7 @@
       </c>
       <c r="B752" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -9472,7 +9460,7 @@
       </c>
       <c r="B754" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -9520,7 +9508,7 @@
       </c>
       <c r="B758" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -9652,7 +9640,7 @@
       </c>
       <c r="B769" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -9832,7 +9820,7 @@
       </c>
       <c r="B784" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -9940,7 +9928,7 @@
       </c>
       <c r="B793" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -10072,7 +10060,7 @@
       </c>
       <c r="B804" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -10120,7 +10108,7 @@
       </c>
       <c r="B808" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -10144,7 +10132,7 @@
       </c>
       <c r="B810" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -10252,7 +10240,7 @@
       </c>
       <c r="B819" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -10420,7 +10408,7 @@
       </c>
       <c r="B833" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -10492,7 +10480,7 @@
       </c>
       <c r="B839" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -10504,7 +10492,7 @@
       </c>
       <c r="B840" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -10552,7 +10540,7 @@
       </c>
       <c r="B844" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -10636,7 +10624,7 @@
       </c>
       <c r="B851" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -10720,7 +10708,7 @@
       </c>
       <c r="B858" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -10900,7 +10888,7 @@
       </c>
       <c r="B873" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -11032,7 +11020,7 @@
       </c>
       <c r="B884" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -11224,7 +11212,7 @@
       </c>
       <c r="B900" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>

</xml_diff>